<commit_message>
docs: add seed user credentials Excel file
</commit_message>
<xml_diff>
--- a/docs/Gizera_Seed_Credentials.xlsx
+++ b/docs/Gizera_Seed_Credentials.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Credential Users" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="User Credentials" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,10 +28,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -52,20 +52,68 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFE8D6"/>
+        <bgColor rgb="00FFE8D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6F5E0"/>
+        <bgColor rgb="00D6F5E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E8FF"/>
+        <bgColor rgb="00D6E8FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F0D6"/>
+        <bgColor rgb="00F5F0D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD6D6"/>
+        <bgColor rgb="00FFD6D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8D6FF"/>
+        <bgColor rgb="00E8D6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6FFF5"/>
+        <bgColor rgb="00D6FFF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
+        <bgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E0F0FF"/>
         <bgColor rgb="00E0F0FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0FFE0"/>
-        <bgColor rgb="00E0FFE0"/>
+        <fgColor rgb="00FFF0D6"/>
+        <bgColor rgb="00FFF0D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF0E0"/>
-        <bgColor rgb="00FFF0E0"/>
+        <fgColor rgb="00F0D6FF"/>
+        <bgColor rgb="00F0D6FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -87,10 +135,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -100,10 +148,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -112,6 +156,38 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -477,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -486,6 +562,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -519,6 +596,11 @@
           <t>Password</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>No. Telepon</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -549,6 +631,11 @@
           <t>superadmin123</t>
         </is>
       </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -579,6 +666,11 @@
           <t>password123</t>
         </is>
       </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n">
@@ -609,6 +701,11 @@
           <t>password123</t>
         </is>
       </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>081234567001</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
@@ -639,394 +736,464 @@
           <t>password123</t>
         </is>
       </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>081234567002</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>PG001</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>budi.santoso@sppg.com</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Budi Santoso</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>pengadaan</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>081234567003</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>PG002</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>rina.wati@sppg.com</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Rina Wati</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>pengadaan</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>081234567004</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>AK001</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>ahmad.fauzi@sppg.com</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>Ahmad Fauzi</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>akuntan</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>081234567005</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>CH001</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>rudi.hermawan@sppg.com</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Rudi Hermawan</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>chef</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>081234567006</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>CH002</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>yanti.susanti@sppg.com</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Yanti Susanti</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>chef</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>081234567007</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>PK001</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>hendra.gunawan@sppg.com</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>Hendra Gunawan</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>packing</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>081234567008</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>PK002</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>lina.marlina@sppg.com</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Lina Marlina</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>packing</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>081234567009</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>DR001</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>joko.widodo@sppg.com</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>Joko Widodo</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>driver</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>081234567010</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>DR002</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>agus.setiawan@sppg.com</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>Agus Setiawan</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>driver</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>081234567011</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>AL001</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="19" t="inlineStr">
         <is>
           <t>dian.permata@sppg.com</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>Dian Permata</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="19" t="inlineStr">
         <is>
           <t>asisten_lapangan</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>081234567012</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>KB001</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>sri.wahyuni@sppg.com</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>Sri Wahyuni</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>kebersihan</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="inlineStr">
+        <is>
+          <t>081234567013</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="n">
+      <c r="A17" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>KY001</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="23" t="inlineStr">
         <is>
           <t>prof.suharno@yayasan.com</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="23" t="inlineStr">
         <is>
           <t>Prof. Suharno</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="23" t="inlineStr">
         <is>
           <t>kepala_yayasan</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="inlineStr">
+        <is>
+          <t>081234567014</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n">
+      <c r="A18" s="24" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="25" t="inlineStr">
         <is>
           <t>AB001</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="25" t="inlineStr">
         <is>
           <t>admin.bgn@bgn.go.id</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="25" t="inlineStr">
         <is>
           <t>Dr. Bambang Sutrisno</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E18" s="25" t="inlineStr">
         <is>
           <t>admin_bgn</t>
         </is>
       </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>password123</t>
+      <c r="F18" s="25" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="G18" s="25" t="inlineStr">
+        <is>
+          <t>081234567015</t>
         </is>
       </c>
     </row>

</xml_diff>